<commit_message>
Added Process review document
</commit_message>
<xml_diff>
--- a/COTs_Export_Merged_Docs/WorkFlows/Workflow Steps/Execution_Operation_Processes_Steps.xlsx
+++ b/COTs_Export_Merged_Docs/WorkFlows/Workflow Steps/Execution_Operation_Processes_Steps.xlsx
@@ -5,12 +5,12 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\arman.buena\Downloads\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\arman.buena\Desktop\COTS\COTS_GitRepo\COTS\COTs_Export_Merged_Docs\WorkFlows\Workflow Steps\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A67BC7D0-9253-401B-9C73-A29A16100B82}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{881AEC92-5200-4EC9-AC68-62C5EB67B070}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="19090" yWindow="-110" windowWidth="19420" windowHeight="10300" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Detailed Process" sheetId="1" r:id="rId1"/>
@@ -25,6 +25,30 @@
 </workbook>
 </file>
 
+<file path=xl/comments1.xml><?xml version="1.0" encoding="utf-8"?>
+<comments xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr">
+  <authors>
+    <author>Arman Buenaventura</author>
+  </authors>
+  <commentList>
+    <comment ref="A26" authorId="0" shapeId="0" xr:uid="{6061BD79-EBEE-43B0-8022-F4264664F113}">
+      <text>
+        <r>
+          <rPr>
+            <b/>
+            <sz val="9"/>
+            <color indexed="81"/>
+            <rFont val="Tahoma"/>
+            <charset val="1"/>
+          </rPr>
+          <t>Missing screen</t>
+        </r>
+      </text>
+    </comment>
+  </commentList>
+</comments>
+</file>
+
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
 <sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1034" uniqueCount="380">
   <si>
@@ -1172,7 +1196,7 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="16" x14ac:knownFonts="1">
+  <fonts count="17" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -1264,8 +1288,15 @@
       <name val="Arial"/>
       <family val="2"/>
     </font>
+    <font>
+      <b/>
+      <sz val="9"/>
+      <color indexed="81"/>
+      <name val="Tahoma"/>
+      <charset val="1"/>
+    </font>
   </fonts>
-  <fills count="12">
+  <fills count="13">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -1320,6 +1351,12 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="FFD9E2F3"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFFF00"/>
+        <bgColor indexed="64"/>
       </patternFill>
     </fill>
   </fills>
@@ -1424,7 +1461,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="37">
+  <cellXfs count="40">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="3" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -1477,26 +1514,22 @@
     <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="7" fillId="6" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="7" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="4" fillId="11" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="4" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="4" fillId="11" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="7" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="7" fillId="6" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="3" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="15" fillId="6" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
@@ -1505,6 +1538,19 @@
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="12" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="12" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="12" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -1807,7 +1853,7 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:M69"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
@@ -1824,36 +1870,36 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:13" ht="16.8" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A1" s="28" t="s">
+      <c r="A1" s="30" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="29"/>
-      <c r="C1" s="29"/>
-      <c r="D1" s="29"/>
-      <c r="E1" s="29"/>
+      <c r="B1" s="31"/>
+      <c r="C1" s="31"/>
+      <c r="D1" s="31"/>
+      <c r="E1" s="31"/>
     </row>
     <row r="2" spans="1:13" x14ac:dyDescent="0.3">
-      <c r="A2" s="30" t="s">
+      <c r="A2" s="35" t="s">
         <v>1</v>
       </c>
-      <c r="B2" s="29"/>
-      <c r="C2" s="29"/>
-      <c r="D2" s="29"/>
-      <c r="E2" s="29"/>
+      <c r="B2" s="31"/>
+      <c r="C2" s="31"/>
+      <c r="D2" s="31"/>
+      <c r="E2" s="31"/>
     </row>
     <row r="3" spans="1:13" ht="49.2" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="F3" s="34" t="s">
+      <c r="F3" s="32" t="s">
         <v>379</v>
       </c>
-      <c r="G3" s="35"/>
-      <c r="H3" s="35"/>
-      <c r="I3" s="35"/>
-      <c r="J3" s="36"/>
-      <c r="K3" s="31" t="s">
+      <c r="G3" s="33"/>
+      <c r="H3" s="33"/>
+      <c r="I3" s="33"/>
+      <c r="J3" s="34"/>
+      <c r="K3" s="22" t="s">
         <v>3</v>
       </c>
-      <c r="L3" s="26"/>
-      <c r="M3" s="32"/>
+      <c r="L3" s="23"/>
+      <c r="M3" s="24"/>
     </row>
     <row r="4" spans="1:13" ht="28.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A4" s="2" t="s">
@@ -1897,18 +1943,18 @@
       </c>
     </row>
     <row r="5" spans="1:13" ht="18" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A5" s="22" t="s">
+      <c r="A5" s="27" t="s">
         <v>17</v>
       </c>
-      <c r="B5" s="23"/>
-      <c r="C5" s="23"/>
-      <c r="D5" s="23"/>
-      <c r="E5" s="24"/>
+      <c r="B5" s="28"/>
+      <c r="C5" s="28"/>
+      <c r="D5" s="28"/>
+      <c r="E5" s="29"/>
       <c r="F5" s="25"/>
-      <c r="G5" s="26"/>
-      <c r="H5" s="26"/>
-      <c r="I5" s="26"/>
-      <c r="J5" s="27"/>
+      <c r="G5" s="23"/>
+      <c r="H5" s="23"/>
+      <c r="I5" s="23"/>
+      <c r="J5" s="26"/>
       <c r="K5" s="18"/>
       <c r="L5" s="18"/>
       <c r="M5" s="18"/>
@@ -2078,18 +2124,18 @@
       </c>
     </row>
     <row r="10" spans="1:13" ht="18" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A10" s="22" t="s">
+      <c r="A10" s="27" t="s">
         <v>45</v>
       </c>
-      <c r="B10" s="23"/>
-      <c r="C10" s="23"/>
-      <c r="D10" s="23"/>
-      <c r="E10" s="24"/>
+      <c r="B10" s="28"/>
+      <c r="C10" s="28"/>
+      <c r="D10" s="28"/>
+      <c r="E10" s="29"/>
       <c r="F10" s="25"/>
-      <c r="G10" s="26"/>
-      <c r="H10" s="26"/>
-      <c r="I10" s="26"/>
-      <c r="J10" s="27"/>
+      <c r="G10" s="23"/>
+      <c r="H10" s="23"/>
+      <c r="I10" s="23"/>
+      <c r="J10" s="26"/>
       <c r="K10" s="18"/>
       <c r="L10" s="18"/>
       <c r="M10" s="18"/>
@@ -2464,18 +2510,18 @@
       </c>
     </row>
     <row r="20" spans="1:13" ht="18" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A20" s="22" t="s">
+      <c r="A20" s="27" t="s">
         <v>84</v>
       </c>
-      <c r="B20" s="23"/>
-      <c r="C20" s="23"/>
-      <c r="D20" s="23"/>
-      <c r="E20" s="24"/>
+      <c r="B20" s="28"/>
+      <c r="C20" s="28"/>
+      <c r="D20" s="28"/>
+      <c r="E20" s="29"/>
       <c r="F20" s="25"/>
-      <c r="G20" s="26"/>
-      <c r="H20" s="26"/>
-      <c r="I20" s="26"/>
-      <c r="J20" s="27"/>
+      <c r="G20" s="23"/>
+      <c r="H20" s="23"/>
+      <c r="I20" s="23"/>
+      <c r="J20" s="26"/>
       <c r="K20" s="18"/>
       <c r="L20" s="18"/>
       <c r="M20" s="18"/>
@@ -2686,19 +2732,19 @@
       </c>
     </row>
     <row r="26" spans="1:13" ht="22.8" x14ac:dyDescent="0.3">
-      <c r="A26" s="3" t="s">
+      <c r="A26" s="37" t="s">
         <v>106</v>
       </c>
-      <c r="B26" s="4" t="s">
+      <c r="B26" s="38" t="s">
         <v>86</v>
       </c>
-      <c r="C26" s="5" t="s">
+      <c r="C26" s="39" t="s">
         <v>107</v>
       </c>
-      <c r="D26" s="4" t="s">
-        <v>27</v>
-      </c>
-      <c r="E26" s="4" t="s">
+      <c r="D26" s="38" t="s">
+        <v>27</v>
+      </c>
+      <c r="E26" s="38" t="s">
         <v>108</v>
       </c>
       <c r="F26" s="15" t="s">
@@ -2768,18 +2814,18 @@
       </c>
     </row>
     <row r="28" spans="1:13" ht="18" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A28" s="22" t="s">
+      <c r="A28" s="27" t="s">
         <v>117</v>
       </c>
-      <c r="B28" s="23"/>
-      <c r="C28" s="23"/>
-      <c r="D28" s="23"/>
-      <c r="E28" s="24"/>
+      <c r="B28" s="28"/>
+      <c r="C28" s="28"/>
+      <c r="D28" s="28"/>
+      <c r="E28" s="29"/>
       <c r="F28" s="25"/>
-      <c r="G28" s="26"/>
-      <c r="H28" s="26"/>
-      <c r="I28" s="26"/>
-      <c r="J28" s="27"/>
+      <c r="G28" s="23"/>
+      <c r="H28" s="23"/>
+      <c r="I28" s="23"/>
+      <c r="J28" s="26"/>
       <c r="K28" s="18"/>
       <c r="L28" s="18"/>
       <c r="M28" s="18"/>
@@ -3154,18 +3200,18 @@
       </c>
     </row>
     <row r="38" spans="1:13" ht="18" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A38" s="22" t="s">
+      <c r="A38" s="27" t="s">
         <v>160</v>
       </c>
-      <c r="B38" s="23"/>
-      <c r="C38" s="23"/>
-      <c r="D38" s="23"/>
-      <c r="E38" s="24"/>
+      <c r="B38" s="28"/>
+      <c r="C38" s="28"/>
+      <c r="D38" s="28"/>
+      <c r="E38" s="29"/>
       <c r="F38" s="25"/>
-      <c r="G38" s="26"/>
-      <c r="H38" s="26"/>
-      <c r="I38" s="26"/>
-      <c r="J38" s="27"/>
+      <c r="G38" s="23"/>
+      <c r="H38" s="23"/>
+      <c r="I38" s="23"/>
+      <c r="J38" s="26"/>
       <c r="K38" s="18"/>
       <c r="L38" s="18"/>
       <c r="M38" s="18"/>
@@ -3376,18 +3422,18 @@
       </c>
     </row>
     <row r="44" spans="1:13" ht="18" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A44" s="22" t="s">
+      <c r="A44" s="27" t="s">
         <v>180</v>
       </c>
-      <c r="B44" s="23"/>
-      <c r="C44" s="23"/>
-      <c r="D44" s="23"/>
-      <c r="E44" s="24"/>
+      <c r="B44" s="28"/>
+      <c r="C44" s="28"/>
+      <c r="D44" s="28"/>
+      <c r="E44" s="29"/>
       <c r="F44" s="25"/>
-      <c r="G44" s="26"/>
-      <c r="H44" s="26"/>
-      <c r="I44" s="26"/>
-      <c r="J44" s="27"/>
+      <c r="G44" s="23"/>
+      <c r="H44" s="23"/>
+      <c r="I44" s="23"/>
+      <c r="J44" s="26"/>
       <c r="K44" s="18"/>
       <c r="L44" s="18"/>
       <c r="M44" s="18"/>
@@ -3434,18 +3480,18 @@
       </c>
     </row>
     <row r="46" spans="1:13" ht="18" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A46" s="22" t="s">
+      <c r="A46" s="27" t="s">
         <v>184</v>
       </c>
-      <c r="B46" s="23"/>
-      <c r="C46" s="23"/>
-      <c r="D46" s="23"/>
-      <c r="E46" s="24"/>
+      <c r="B46" s="28"/>
+      <c r="C46" s="28"/>
+      <c r="D46" s="28"/>
+      <c r="E46" s="29"/>
       <c r="F46" s="25"/>
-      <c r="G46" s="26"/>
-      <c r="H46" s="26"/>
-      <c r="I46" s="26"/>
-      <c r="J46" s="27"/>
+      <c r="G46" s="23"/>
+      <c r="H46" s="23"/>
+      <c r="I46" s="23"/>
+      <c r="J46" s="26"/>
       <c r="K46" s="18"/>
       <c r="L46" s="18"/>
       <c r="M46" s="18"/>
@@ -3738,18 +3784,18 @@
       </c>
     </row>
     <row r="54" spans="1:13" ht="18" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A54" s="22" t="s">
+      <c r="A54" s="27" t="s">
         <v>206</v>
       </c>
-      <c r="B54" s="23"/>
-      <c r="C54" s="23"/>
-      <c r="D54" s="23"/>
-      <c r="E54" s="24"/>
+      <c r="B54" s="28"/>
+      <c r="C54" s="28"/>
+      <c r="D54" s="28"/>
+      <c r="E54" s="29"/>
       <c r="F54" s="25"/>
-      <c r="G54" s="26"/>
-      <c r="H54" s="26"/>
-      <c r="I54" s="26"/>
-      <c r="J54" s="27"/>
+      <c r="G54" s="23"/>
+      <c r="H54" s="23"/>
+      <c r="I54" s="23"/>
+      <c r="J54" s="26"/>
       <c r="K54" s="18"/>
       <c r="L54" s="18"/>
       <c r="M54" s="18"/>
@@ -3878,18 +3924,18 @@
       </c>
     </row>
     <row r="58" spans="1:13" ht="18" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A58" s="22" t="s">
+      <c r="A58" s="27" t="s">
         <v>216</v>
       </c>
-      <c r="B58" s="23"/>
-      <c r="C58" s="23"/>
-      <c r="D58" s="23"/>
-      <c r="E58" s="24"/>
+      <c r="B58" s="28"/>
+      <c r="C58" s="28"/>
+      <c r="D58" s="28"/>
+      <c r="E58" s="29"/>
       <c r="F58" s="25"/>
-      <c r="G58" s="26"/>
-      <c r="H58" s="26"/>
-      <c r="I58" s="26"/>
-      <c r="J58" s="27"/>
+      <c r="G58" s="23"/>
+      <c r="H58" s="23"/>
+      <c r="I58" s="23"/>
+      <c r="J58" s="26"/>
       <c r="K58" s="18"/>
       <c r="L58" s="18"/>
       <c r="M58" s="18"/>
@@ -3936,18 +3982,18 @@
       </c>
     </row>
     <row r="60" spans="1:13" ht="18" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A60" s="22" t="s">
+      <c r="A60" s="27" t="s">
         <v>220</v>
       </c>
-      <c r="B60" s="23"/>
-      <c r="C60" s="23"/>
-      <c r="D60" s="23"/>
-      <c r="E60" s="24"/>
+      <c r="B60" s="28"/>
+      <c r="C60" s="28"/>
+      <c r="D60" s="28"/>
+      <c r="E60" s="29"/>
       <c r="F60" s="25"/>
-      <c r="G60" s="26"/>
-      <c r="H60" s="26"/>
-      <c r="I60" s="26"/>
-      <c r="J60" s="27"/>
+      <c r="G60" s="23"/>
+      <c r="H60" s="23"/>
+      <c r="I60" s="23"/>
+      <c r="J60" s="26"/>
       <c r="K60" s="18"/>
       <c r="L60" s="18"/>
       <c r="M60" s="18"/>
@@ -4035,18 +4081,18 @@
       </c>
     </row>
     <row r="63" spans="1:13" ht="18" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A63" s="22" t="s">
+      <c r="A63" s="27" t="s">
         <v>230</v>
       </c>
-      <c r="B63" s="23"/>
-      <c r="C63" s="23"/>
-      <c r="D63" s="23"/>
-      <c r="E63" s="24"/>
+      <c r="B63" s="28"/>
+      <c r="C63" s="28"/>
+      <c r="D63" s="28"/>
+      <c r="E63" s="29"/>
       <c r="F63" s="25"/>
-      <c r="G63" s="26"/>
-      <c r="H63" s="26"/>
-      <c r="I63" s="26"/>
-      <c r="J63" s="27"/>
+      <c r="G63" s="23"/>
+      <c r="H63" s="23"/>
+      <c r="I63" s="23"/>
+      <c r="J63" s="26"/>
       <c r="K63" s="18"/>
       <c r="L63" s="18"/>
       <c r="M63" s="18"/>
@@ -4216,18 +4262,18 @@
       </c>
     </row>
     <row r="68" spans="1:13" ht="18" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A68" s="22" t="s">
+      <c r="A68" s="27" t="s">
         <v>243</v>
       </c>
-      <c r="B68" s="23"/>
-      <c r="C68" s="23"/>
-      <c r="D68" s="23"/>
-      <c r="E68" s="24"/>
+      <c r="B68" s="28"/>
+      <c r="C68" s="28"/>
+      <c r="D68" s="28"/>
+      <c r="E68" s="29"/>
       <c r="F68" s="25"/>
-      <c r="G68" s="26"/>
-      <c r="H68" s="26"/>
-      <c r="I68" s="26"/>
-      <c r="J68" s="27"/>
+      <c r="G68" s="23"/>
+      <c r="H68" s="23"/>
+      <c r="I68" s="23"/>
+      <c r="J68" s="26"/>
       <c r="K68" s="18"/>
       <c r="L68" s="18"/>
       <c r="M68" s="18"/>
@@ -4276,14 +4322,14 @@
   </sheetData>
   <autoFilter ref="A4:M69" xr:uid="{00000000-0009-0000-0000-000000000000}"/>
   <mergeCells count="28">
-    <mergeCell ref="K3:M3"/>
-    <mergeCell ref="F58:J58"/>
-    <mergeCell ref="A20:E20"/>
-    <mergeCell ref="A38:E38"/>
-    <mergeCell ref="A10:E10"/>
-    <mergeCell ref="A28:E28"/>
-    <mergeCell ref="A44:E44"/>
-    <mergeCell ref="A58:E58"/>
+    <mergeCell ref="A60:E60"/>
+    <mergeCell ref="F54:J54"/>
+    <mergeCell ref="F10:J10"/>
+    <mergeCell ref="F68:J68"/>
+    <mergeCell ref="F63:J63"/>
+    <mergeCell ref="A68:E68"/>
+    <mergeCell ref="A63:E63"/>
+    <mergeCell ref="F60:J60"/>
     <mergeCell ref="A1:E1"/>
     <mergeCell ref="F3:J3"/>
     <mergeCell ref="A54:E54"/>
@@ -4296,16 +4342,17 @@
     <mergeCell ref="A5:E5"/>
     <mergeCell ref="F46:J46"/>
     <mergeCell ref="F44:J44"/>
-    <mergeCell ref="A60:E60"/>
-    <mergeCell ref="F54:J54"/>
-    <mergeCell ref="F10:J10"/>
-    <mergeCell ref="F68:J68"/>
-    <mergeCell ref="F63:J63"/>
-    <mergeCell ref="A68:E68"/>
-    <mergeCell ref="A63:E63"/>
-    <mergeCell ref="F60:J60"/>
+    <mergeCell ref="K3:M3"/>
+    <mergeCell ref="F58:J58"/>
+    <mergeCell ref="A20:E20"/>
+    <mergeCell ref="A38:E38"/>
+    <mergeCell ref="A10:E10"/>
+    <mergeCell ref="A28:E28"/>
+    <mergeCell ref="A44:E44"/>
+    <mergeCell ref="A58:E58"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <legacyDrawing r:id="rId1"/>
 </worksheet>
 </file>
 
@@ -4324,31 +4371,31 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:10" ht="16.8" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A1" s="28" t="s">
+      <c r="A1" s="30" t="s">
         <v>250</v>
       </c>
-      <c r="B1" s="29"/>
-      <c r="C1" s="29"/>
-      <c r="D1" s="29"/>
-      <c r="E1" s="29"/>
+      <c r="B1" s="31"/>
+      <c r="C1" s="31"/>
+      <c r="D1" s="31"/>
+      <c r="E1" s="31"/>
     </row>
     <row r="2" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="A2" s="30" t="s">
+      <c r="A2" s="35" t="s">
         <v>251</v>
       </c>
-      <c r="B2" s="29"/>
-      <c r="C2" s="29"/>
-      <c r="D2" s="29"/>
-      <c r="E2" s="29"/>
+      <c r="B2" s="31"/>
+      <c r="C2" s="31"/>
+      <c r="D2" s="31"/>
+      <c r="E2" s="31"/>
     </row>
     <row r="3" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="F3" s="33" t="s">
+      <c r="F3" s="36" t="s">
         <v>2</v>
       </c>
-      <c r="G3" s="23"/>
-      <c r="H3" s="23"/>
-      <c r="I3" s="23"/>
-      <c r="J3" s="24"/>
+      <c r="G3" s="28"/>
+      <c r="H3" s="28"/>
+      <c r="I3" s="28"/>
+      <c r="J3" s="29"/>
     </row>
     <row r="4" spans="1:10" ht="28.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A4" s="2" t="s">
@@ -4383,20 +4430,20 @@
       </c>
     </row>
     <row r="5" spans="1:10" ht="18" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A5" s="22" t="s">
+      <c r="A5" s="27" t="s">
         <v>17</v>
       </c>
-      <c r="B5" s="23"/>
-      <c r="C5" s="23"/>
-      <c r="D5" s="23"/>
-      <c r="E5" s="24"/>
-      <c r="F5" s="22" t="s">
+      <c r="B5" s="28"/>
+      <c r="C5" s="28"/>
+      <c r="D5" s="28"/>
+      <c r="E5" s="29"/>
+      <c r="F5" s="27" t="s">
         <v>18</v>
       </c>
-      <c r="G5" s="23"/>
-      <c r="H5" s="23"/>
-      <c r="I5" s="23"/>
-      <c r="J5" s="24"/>
+      <c r="G5" s="28"/>
+      <c r="H5" s="28"/>
+      <c r="I5" s="28"/>
+      <c r="J5" s="29"/>
     </row>
     <row r="6" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A6" s="3" t="s">
@@ -4509,20 +4556,20 @@
       <c r="J10" s="4"/>
     </row>
     <row r="11" spans="1:10" ht="18" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A11" s="22" t="s">
+      <c r="A11" s="27" t="s">
         <v>45</v>
       </c>
-      <c r="B11" s="23"/>
-      <c r="C11" s="23"/>
-      <c r="D11" s="23"/>
-      <c r="E11" s="24"/>
-      <c r="F11" s="22" t="s">
+      <c r="B11" s="28"/>
+      <c r="C11" s="28"/>
+      <c r="D11" s="28"/>
+      <c r="E11" s="29"/>
+      <c r="F11" s="27" t="s">
         <v>18</v>
       </c>
-      <c r="G11" s="23"/>
-      <c r="H11" s="23"/>
-      <c r="I11" s="23"/>
-      <c r="J11" s="24"/>
+      <c r="G11" s="28"/>
+      <c r="H11" s="28"/>
+      <c r="I11" s="28"/>
+      <c r="J11" s="29"/>
     </row>
     <row r="12" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A12" s="6" t="s">
@@ -4811,20 +4858,20 @@
       <c r="J24" s="7"/>
     </row>
     <row r="25" spans="1:10" ht="18" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A25" s="22" t="s">
+      <c r="A25" s="27" t="s">
         <v>267</v>
       </c>
-      <c r="B25" s="23"/>
-      <c r="C25" s="23"/>
-      <c r="D25" s="23"/>
-      <c r="E25" s="24"/>
-      <c r="F25" s="22" t="s">
+      <c r="B25" s="28"/>
+      <c r="C25" s="28"/>
+      <c r="D25" s="28"/>
+      <c r="E25" s="29"/>
+      <c r="F25" s="27" t="s">
         <v>18</v>
       </c>
-      <c r="G25" s="23"/>
-      <c r="H25" s="23"/>
-      <c r="I25" s="23"/>
-      <c r="J25" s="24"/>
+      <c r="G25" s="28"/>
+      <c r="H25" s="28"/>
+      <c r="I25" s="28"/>
+      <c r="J25" s="29"/>
     </row>
     <row r="26" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A26" s="3" t="s">
@@ -5047,20 +5094,20 @@
       <c r="J35" s="4"/>
     </row>
     <row r="36" spans="1:10" ht="18" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A36" s="22" t="s">
+      <c r="A36" s="27" t="s">
         <v>283</v>
       </c>
-      <c r="B36" s="23"/>
-      <c r="C36" s="23"/>
-      <c r="D36" s="23"/>
-      <c r="E36" s="24"/>
-      <c r="F36" s="22" t="s">
+      <c r="B36" s="28"/>
+      <c r="C36" s="28"/>
+      <c r="D36" s="28"/>
+      <c r="E36" s="29"/>
+      <c r="F36" s="27" t="s">
         <v>18</v>
       </c>
-      <c r="G36" s="23"/>
-      <c r="H36" s="23"/>
-      <c r="I36" s="23"/>
-      <c r="J36" s="24"/>
+      <c r="G36" s="28"/>
+      <c r="H36" s="28"/>
+      <c r="I36" s="28"/>
+      <c r="J36" s="29"/>
     </row>
     <row r="37" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A37" s="6" t="s">

</xml_diff>